<commit_message>
Lock Ralph Lauren Boca commercial inputs to Luke's 3 Sep 2026 terms.
Write 21 weeks, 10% CM, 1.5% insurance, $4,400/wk superintendent, and 1% pre-con (first pay app) as SET. Leave trade dollars, parking/shutdown counts, CO markup, weekly GC lump, and the grand total OPEN. Keep confidential / not-a-bid / not-sent-to-Charrette banners and the Heritage Prep RL look.

Co-authored-by: lucasoffice <lucasoffice@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ralph-lauren/boca/RL_Boca_CostPlus_GC.xlsx
+++ b/ralph-lauren/boca/RL_Boca_CostPlus_GC.xlsx
@@ -15,6 +15,7 @@
   </sheets>
   <definedNames>
     <definedName name="Weeks">'LANDIS FORM'!$B$5</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="5">'PROPOSED ROSTER'!$A$1:$E$26</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'COVER'!$A$1:$E$28</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'GC BID FORM'!$A$9:$K$80</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'LANDIS FORM'!$B$19:$D$39</definedName>
@@ -169,7 +170,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -229,8 +230,20 @@
         <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6E3F0"/>
+        <bgColor rgb="00D6E3F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE599"/>
+        <bgColor rgb="00FFE599"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -267,11 +280,55 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="109">
+  <cellXfs count="123">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -527,6 +584,38 @@
     <xf numFmtId="0" fontId="9" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="12" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="12" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="13" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -814,14 +903,14 @@
     <row r="4" ht="20" customHeight="1">
       <c r="B4" s="76" t="inlineStr">
         <is>
-          <t>This is a first-draft open-book exhibit, not a lump-sum bid.</t>
+          <t>This is an open-book exhibit after Luke’s 3 Sep 2026 lock, not a lump-sum bid.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="36" customHeight="1">
       <c r="B5" s="30" t="inlineStr">
         <is>
-          <t>Cost-plus CM + GC. Yellow cells on the following sheets are commercial inputs still OPEN. No weeks, CM fee %, insurance %, weekly superintendent rate, or job grand total has been filled as a decided number.</t>
+          <t>Cost-plus CM + GC. SET: 21 weeks, 10% CM fee, 1.5% insurance, $4,400/wk superintendent, 1% pre-construction (first pay app / NTP). Still OPEN: trade dollars, weekly GC lump, CO markup %, parking months, sprinkler-shutdown count, pre-con dollars, grand total. Not a send to Charrette.</t>
         </is>
       </c>
     </row>
@@ -831,9 +920,6 @@
           <t>JOB IDENTITY</t>
         </is>
       </c>
-      <c r="C7" s="42" t="n"/>
-      <c r="D7" s="42" t="n"/>
-      <c r="E7" s="42" t="n"/>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="B8" s="77" t="inlineStr">
@@ -846,8 +932,8 @@
           <t>Ralph Lauren</t>
         </is>
       </c>
-      <c r="D8" s="79" t="n"/>
-      <c r="E8" s="79" t="n"/>
+      <c r="D8" s="109" t="n"/>
+      <c r="E8" s="110" t="n"/>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="B9" s="77" t="inlineStr">
@@ -860,8 +946,8 @@
           <t>Town Center at Boca Raton, Simon space 1062, 600 Glades Road</t>
         </is>
       </c>
-      <c r="D9" s="79" t="n"/>
-      <c r="E9" s="79" t="n"/>
+      <c r="D9" s="109" t="n"/>
+      <c r="E9" s="110" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="B10" s="77" t="inlineStr">
@@ -874,8 +960,8 @@
           <t>3,384 sf</t>
         </is>
       </c>
-      <c r="D10" s="79" t="n"/>
-      <c r="E10" s="79" t="n"/>
+      <c r="D10" s="109" t="n"/>
+      <c r="E10" s="110" t="n"/>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="B11" s="77" t="inlineStr">
@@ -888,8 +974,8 @@
           <t>Charrette MG — Landis Kauffman, Claudia Mardones</t>
         </is>
       </c>
-      <c r="D11" s="79" t="n"/>
-      <c r="E11" s="79" t="n"/>
+      <c r="D11" s="109" t="n"/>
+      <c r="E11" s="110" t="n"/>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="B12" s="77" t="inlineStr">
@@ -902,8 +988,8 @@
           <t>Cost-plus / CM + GC  (not lump sum)</t>
         </is>
       </c>
-      <c r="D12" s="79" t="n"/>
-      <c r="E12" s="79" t="n"/>
+      <c r="D12" s="109" t="n"/>
+      <c r="E12" s="110" t="n"/>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="B13" s="77" t="inlineStr">
@@ -916,8 +1002,8 @@
           <t>Ralph Lauren policy: net 90</t>
         </is>
       </c>
-      <c r="D13" s="79" t="n"/>
-      <c r="E13" s="79" t="n"/>
+      <c r="D13" s="109" t="n"/>
+      <c r="E13" s="110" t="n"/>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="B14" s="77" t="inlineStr">
@@ -930,8 +1016,8 @@
           <t>Commence 2027-04-02  |  Substantial 2027-08-18 (~19.5 weeks)  |  Final 2027-08-25</t>
         </is>
       </c>
-      <c r="D14" s="79" t="n"/>
-      <c r="E14" s="79" t="n"/>
+      <c r="D14" s="109" t="n"/>
+      <c r="E14" s="110" t="n"/>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="B15" s="77" t="inlineStr">
@@ -944,8 +1030,8 @@
           <t>TPG</t>
         </is>
       </c>
-      <c r="D15" s="79" t="n"/>
-      <c r="E15" s="79" t="n"/>
+      <c r="D15" s="109" t="n"/>
+      <c r="E15" s="110" t="n"/>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="B16" s="77" t="inlineStr">
@@ -958,8 +1044,8 @@
           <t>2026-07-14</t>
         </is>
       </c>
-      <c r="D16" s="79" t="n"/>
-      <c r="E16" s="79" t="n"/>
+      <c r="D16" s="109" t="n"/>
+      <c r="E16" s="110" t="n"/>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="B17" s="77" t="inlineStr">
@@ -972,8 +1058,8 @@
           <t>dorit.alexander@ralphlauren.com</t>
         </is>
       </c>
-      <c r="D17" s="79" t="n"/>
-      <c r="E17" s="79" t="n"/>
+      <c r="D17" s="109" t="n"/>
+      <c r="E17" s="110" t="n"/>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="B18" s="77" t="inlineStr">
@@ -986,8 +1072,8 @@
           <t>Excluded / invoiced separately</t>
         </is>
       </c>
-      <c r="D18" s="79" t="n"/>
-      <c r="E18" s="79" t="n"/>
+      <c r="D18" s="109" t="n"/>
+      <c r="E18" s="110" t="n"/>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="B19" s="77" t="inlineStr">
@@ -1000,8 +1086,8 @@
           <t>Invoiced separately</t>
         </is>
       </c>
-      <c r="D19" s="79" t="n"/>
-      <c r="E19" s="79" t="n"/>
+      <c r="D19" s="109" t="n"/>
+      <c r="E19" s="110" t="n"/>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="B20" s="77" t="inlineStr">
@@ -1014,8 +1100,8 @@
           <t>LUX Brand Company</t>
         </is>
       </c>
-      <c r="D20" s="79" t="n"/>
-      <c r="E20" s="79" t="n"/>
+      <c r="D20" s="109" t="n"/>
+      <c r="E20" s="110" t="n"/>
     </row>
     <row r="22">
       <c r="B22" s="42" t="inlineStr">
@@ -1023,9 +1109,6 @@
           <t>NOTES</t>
         </is>
       </c>
-      <c r="C22" s="42" t="n"/>
-      <c r="D22" s="42" t="n"/>
-      <c r="E22" s="42" t="n"/>
     </row>
     <row r="23" ht="42" customHeight="1">
       <c r="B23" s="80" t="inlineStr">
@@ -1035,25 +1118,25 @@
       </c>
       <c r="C23" s="81" t="inlineStr">
         <is>
-          <t>This workbook is a first-draft open-book CM exhibit for discussion with Charrette. It is not a lump-sum bid and not an awarded contract price.</t>
-        </is>
-      </c>
-      <c r="D23" s="79" t="n"/>
-      <c r="E23" s="79" t="n"/>
+          <t>This workbook is an open-book CM exhibit for internal review after Luke’s 3 Sep 2026 lock. It is not a lump-sum bid, not an awarded contract price, and not a send to Charrette.</t>
+        </is>
+      </c>
+      <c r="D23" s="109" t="n"/>
+      <c r="E23" s="110" t="n"/>
     </row>
     <row r="24" ht="42" customHeight="1">
       <c r="B24" s="80" t="inlineStr">
         <is>
-          <t>Blank inputs</t>
+          <t>Luke lock / remaining blanks</t>
         </is>
       </c>
       <c r="C24" s="81" t="inlineStr">
         <is>
-          <t>Weeks, CM fee %, insurance %, and weekly superintendent stay blank (yellow) until confirmed. Do not read $0 rollups on GC BID FORM or LANDIS FORM as a bid total.</t>
-        </is>
-      </c>
-      <c r="D24" s="79" t="n"/>
-      <c r="E24" s="79" t="n"/>
+          <t>Luke lock 3 Sep 2026 filled duration, CM fee %, insurance %, and weekly superintendent. Do not read $0 rollups on GC BID FORM or LANDIS FORM as a bid total — trades are unbid.</t>
+        </is>
+      </c>
+      <c r="D24" s="109" t="n"/>
+      <c r="E24" s="110" t="n"/>
     </row>
     <row r="25" ht="42" customHeight="1">
       <c r="B25" s="80" t="inlineStr">
@@ -1063,11 +1146,11 @@
       </c>
       <c r="C25" s="81" t="inlineStr">
         <is>
-          <t>Intake calendar is commence 2027-04-02 through substantial 2027-08-18 (~19.5 weeks), final 2027-08-25. A leftover 13-week figure from a prior template is listed on OPEN ITEMS and is not used as the duration.</t>
-        </is>
-      </c>
-      <c r="D25" s="79" t="n"/>
-      <c r="E25" s="79" t="n"/>
+          <t>Intake calendar is commence 2027-04-02 through substantial 2027-08-18 (~19.5 weeks), final 2027-08-25. Luke locked 21 weeks for the fee form (reconciles 19.5 vs the 20–23 band). The leftover 13-week figure is not used.</t>
+        </is>
+      </c>
+      <c r="D25" s="109" t="n"/>
+      <c r="E25" s="110" t="n"/>
     </row>
     <row r="26" ht="42" customHeight="1">
       <c r="B26" s="80" t="inlineStr">
@@ -1080,8 +1163,8 @@
           <t>Permit fees are excluded and invoiced separately. Sales tax is invoiced separately.</t>
         </is>
       </c>
-      <c r="D26" s="79" t="n"/>
-      <c r="E26" s="79" t="n"/>
+      <c r="D26" s="109" t="n"/>
+      <c r="E26" s="110" t="n"/>
     </row>
     <row r="27" ht="42" customHeight="1">
       <c r="B27" s="80" t="inlineStr">
@@ -1091,11 +1174,11 @@
       </c>
       <c r="C27" s="81" t="inlineStr">
         <is>
-          <t>No trade-package dollars are entered. PROPOSED ROSTER is proposed, not awarded. Mall unit rates are listed on MALL FEES; parking months and sprinkler-shutdown count stay OPEN.</t>
-        </is>
-      </c>
-      <c r="D27" s="79" t="n"/>
-      <c r="E27" s="79" t="n"/>
+          <t>No trade-package dollars are entered. PROPOSED ROSTER is proposed, not awarded (Robert Colvin proposed, not awarded). Mall unit rates are listed on MALL FEES; parking months and sprinkler-shutdown count stay OPEN.</t>
+        </is>
+      </c>
+      <c r="D27" s="109" t="n"/>
+      <c r="E27" s="110" t="n"/>
     </row>
     <row r="28" ht="42" customHeight="1">
       <c r="B28" s="80" t="inlineStr">
@@ -1108,8 +1191,8 @@
           <t>COVER  |  GC BID FORM  |  LANDIS FORM  |  OPEN ITEMS  |  MALL FEES  |  PROPOSED ROSTER</t>
         </is>
       </c>
-      <c r="D28" s="79" t="n"/>
-      <c r="E28" s="79" t="n"/>
+      <c r="D28" s="109" t="n"/>
+      <c r="E28" s="110" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="25">
@@ -1185,7 +1268,7 @@
     <row r="10">
       <c r="I10" s="82" t="inlineStr">
         <is>
-          <t>First-draft open-book exhibit — not a lump-sum bid</t>
+          <t>Open-book exhibit after Luke lock 3 Sep 2026 — not a lump-sum bid. Not a send to Charrette.</t>
         </is>
       </c>
     </row>
@@ -1206,7 +1289,7 @@
       </c>
       <c r="K14" s="83" t="inlineStr">
         <is>
-          <t>OPEN — rollup follows blank commercial inputs. Not a lump-sum bid total.</t>
+          <t>Not a lump-sum bid total. Trades unbid. Weekly GC lump still OPEN. Super $4,400 × 21 is on C-6 only.</t>
         </is>
       </c>
     </row>
@@ -1538,14 +1621,16 @@
         <f>J35+J40+J52</f>
         <v/>
       </c>
-      <c r="I33" s="84" t="n"/>
+      <c r="I33" s="111" t="n">
+        <v>0.1</v>
+      </c>
       <c r="J33" s="28">
         <f>H33*I33</f>
         <v/>
       </c>
       <c r="K33" s="83" t="inlineStr">
         <is>
-          <t>OPEN — CM fee / OH&amp;P % not set.</t>
+          <t>SET — Luke locked 10% CM / OH&amp;P on 3 Sep 2026.</t>
         </is>
       </c>
     </row>
@@ -1611,14 +1696,16 @@
         <f>J40+J52+J36</f>
         <v/>
       </c>
-      <c r="I37" s="84" t="n"/>
+      <c r="I37" s="111" t="n">
+        <v>0.015</v>
+      </c>
       <c r="J37" s="28">
         <f>H37*I37</f>
         <v/>
       </c>
       <c r="K37" s="83" t="inlineStr">
         <is>
-          <t>OPEN — insurance % not set.</t>
+          <t>SET — 1.5% liability insurance confirmed (limits confirmed). Workers’ compensation 1.2% is C-7 only; do not double-count into this line.</t>
         </is>
       </c>
     </row>
@@ -1758,7 +1845,7 @@
       </c>
       <c r="K44" s="83" t="inlineStr">
         <is>
-          <t>OPEN — weeks not set. See OPEN ITEMS (duration).</t>
+          <t>OPEN — laborer weeks not set. Job duration is 21 weeks; do not invent a laborer count.</t>
         </is>
       </c>
     </row>
@@ -1929,13 +2016,17 @@
           <t>Superintendent</t>
         </is>
       </c>
-      <c r="E49" s="44" t="n"/>
+      <c r="E49" s="112" t="n">
+        <v>4400</v>
+      </c>
       <c r="F49" s="20" t="inlineStr">
         <is>
           <t>Per Week</t>
         </is>
       </c>
-      <c r="G49" s="39" t="n"/>
+      <c r="G49" s="113" t="n">
+        <v>21</v>
+      </c>
       <c r="H49" s="20" t="inlineStr">
         <is>
           <t>Weeks</t>
@@ -1952,7 +2043,7 @@
       </c>
       <c r="K49" s="83" t="inlineStr">
         <is>
-          <t>OPEN — weekly super rate and weeks not set. See OPEN ITEMS.</t>
+          <t>SET — $4,400/wk × 21 weeks (Luke 3 Sep 2026). Robert Colvin proposed, not awarded. Prior $4,300 / $5,800 figures superseded.</t>
         </is>
       </c>
     </row>
@@ -1992,6 +2083,11 @@
       <c r="J50" s="28">
         <f>E50*J42</f>
         <v/>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>1.2% of payroll subtotal. Separate from B-3 insurance 1.5% — do not double-count.</t>
+        </is>
       </c>
     </row>
     <row r="52">
@@ -2657,12 +2753,14 @@
     <row r="4">
       <c r="B4" s="38" t="inlineStr">
         <is>
-          <t>Duration (weeks) — OPEN, not filled</t>
+          <t>Duration (weeks) — SET 21</t>
         </is>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1">
-      <c r="B5" s="39" t="n"/>
+      <c r="B5" s="113" t="n">
+        <v>21</v>
+      </c>
       <c r="C5" s="40" t="inlineStr">
         <is>
           <t>Weeks (single duration input for this form)</t>
@@ -2670,19 +2768,16 @@
       </c>
       <c r="G5" s="83" t="inlineStr">
         <is>
-          <t>OPEN — leftover 13 weeks not copied. Calendar ~19.5 weeks is on COVER / OPEN ITEMS, not entered here.</t>
+          <t>SET — Luke locked 21 weeks on 3 Sep 2026. RL calendar 2027-04-02 to 2027-08-18 is ~19.5 weeks; 21 reconciles that vs the 20–23 band.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="41" t="inlineStr">
         <is>
-          <t>COMMERCIAL INPUTS (yellow) — blank until confirmed. Leftover template % not copied.</t>
-        </is>
-      </c>
-      <c r="C7" s="42" t="n"/>
-      <c r="D7" s="42" t="n"/>
-      <c r="E7" s="42" t="n"/>
+          <t>COMMERCIAL INPUTS — SET cells filled from Luke lock 3 Sep 2026. Yellow remains OPEN.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="C8" s="88" t="inlineStr">
@@ -2704,13 +2799,13 @@
     <row r="9">
       <c r="C9" s="40" t="inlineStr">
         <is>
-          <t>Pre-construction fee $</t>
+          <t>Pre-construction fee (1% of project total)</t>
         </is>
       </c>
       <c r="E9" s="44" t="n"/>
       <c r="G9" s="83" t="inlineStr">
         <is>
-          <t>OPEN — not set.</t>
+          <t>SET as 1% of project total, payable with first pay application / NTP (not end of job). Dollar cell stays blank until trades are bid.</t>
         </is>
       </c>
     </row>
@@ -2723,7 +2818,7 @@
       <c r="E11" s="44" t="n"/>
       <c r="G11" s="83" t="inlineStr">
         <is>
-          <t>OPEN — weekly GC not set. Super $4,300 / $5,800 not copied.</t>
+          <t>OPEN — weekly GC lump not set as a single dollar. Superintendent breakout is $4,400/wk SET (GC BID FORM C-6). Do not copy $4,400 here as the full lump.</t>
         </is>
       </c>
     </row>
@@ -2733,10 +2828,12 @@
           <t>CM Fee % of cost of work</t>
         </is>
       </c>
-      <c r="E12" s="46" t="n"/>
+      <c r="E12" s="114" t="n">
+        <v>0.1</v>
+      </c>
       <c r="G12" s="83" t="inlineStr">
         <is>
-          <t>OPEN — leftover 10% not copied.</t>
+          <t>SET — Luke locked 10% on 3 Sep 2026.</t>
         </is>
       </c>
     </row>
@@ -2746,26 +2843,25 @@
           <t>Insurance %</t>
         </is>
       </c>
-      <c r="E13" s="46" t="n"/>
+      <c r="E13" s="114" t="n">
+        <v>0.015</v>
+      </c>
       <c r="G13" s="83" t="inlineStr">
         <is>
-          <t>OPEN — leftover 1.5% and Shawn 2%? not copied.</t>
+          <t>SET — working assumption became confirmed 1.5% (limits confirmed). WC 1.2% is on GC BID FORM C-7; not included here.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="C15" s="40" t="inlineStr">
         <is>
-          <t>CO CM Fee % (follows project CM fee)</t>
-        </is>
-      </c>
-      <c r="E15" s="47">
-        <f>E12</f>
-        <v/>
-      </c>
+          <t>CO markup % (separate from project CM fee)</t>
+        </is>
+      </c>
+      <c r="E15" s="115" t="n"/>
       <c r="G15" s="48" t="inlineStr">
         <is>
-          <t>Tracks E12. Stays empty/0 while E12 is OPEN.</t>
+          <t>OPEN — not set. Do not assume equal to the 10% project CM fee.</t>
         </is>
       </c>
     </row>
@@ -2781,7 +2877,7 @@
       </c>
       <c r="G16" s="48" t="inlineStr">
         <is>
-          <t>Tracks E13. Stays empty/0 while E13 is OPEN.</t>
+          <t>Tracks E13 (1.5% insurance). CO markup % above is a separate OPEN line.</t>
         </is>
       </c>
     </row>
@@ -2791,8 +2887,6 @@
           <t>TRADE PACKAGES — no bid packages received; amounts 0</t>
         </is>
       </c>
-      <c r="C18" s="42" t="n"/>
-      <c r="D18" s="42" t="n"/>
     </row>
     <row r="19">
       <c r="B19" s="49" t="inlineStr">
@@ -3083,7 +3177,7 @@
       </c>
       <c r="G40" s="30" t="inlineStr">
         <is>
-          <t>Returns 0 while E11 or B5 is OPEN. Not a decided GC dollar.</t>
+          <t>Returns 0 while weekly GC lump (E11) is OPEN. Super $4,400 × 21 is on GC BID FORM C-6, not this lump.</t>
         </is>
       </c>
     </row>
@@ -3099,7 +3193,7 @@
       </c>
       <c r="G41" s="30" t="inlineStr">
         <is>
-          <t>0 until E12 is set. Leftover 10% not used.</t>
+          <t>CM fee set at 10%. Dollar is 0 while trade packages are $0.</t>
         </is>
       </c>
     </row>
@@ -3115,7 +3209,7 @@
       </c>
       <c r="G42" s="30" t="inlineStr">
         <is>
-          <t>0 until E13 is set. Leftover 1.5% / 2%? not used.</t>
+          <t>Insurance set at 1.5%. Dollar is 0 while trade packages are $0. WC 1.2% is not in this line.</t>
         </is>
       </c>
     </row>
@@ -3125,21 +3219,20 @@
           <t>FORM ROLLUP (not a lump-sum bid)</t>
         </is>
       </c>
-      <c r="C44" s="42" t="n"/>
       <c r="D44" s="59">
         <f>SUM(D20:D42)</f>
         <v/>
       </c>
       <c r="G44" s="83" t="inlineStr">
         <is>
-          <t>OPEN inputs → this rollup is $0. Not a job grand total.</t>
+          <t>Not a job grand total. Trades $0; weekly GC lump OPEN; pre-con dollars OPEN; CO markup OPEN.</t>
         </is>
       </c>
     </row>
     <row r="46" ht="20" customHeight="1">
       <c r="B46" s="60" t="inlineStr">
         <is>
-          <t>Landis-shaped fee form for this cost-plus exhibit. Commercial inputs B5, E9, E11, E12, E13 are blank on purpose. Leftover 10% OH&amp;P, 1.5% insurance, 1% main-office OH, 13 weeks, and super $4,300 / $5,800 are not entered. Trade rows stay $0 until packages are bid. See OPEN ITEMS, MALL FEES, and PROPOSED ROSTER.</t>
+          <t>Landis-shaped fee form after Luke lock 3 Sep 2026. SET: B5 = 21 weeks, E12 = 10% CM, E13 = 1.5% insurance. Pre-con is 1% of project total / first pay app (E9 dollar blank). E11 weekly GC lump and E15 CO markup stay OPEN. Trade rows stay $0 until packages are bid. Not a send to Charrette. See OPEN ITEMS, MALL FEES, and PROPOSED ROSTER.</t>
         </is>
       </c>
     </row>
@@ -3178,7 +3271,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3191,18 +3284,14 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="61" t="inlineStr">
         <is>
-          <t>OPEN ITEMS — first-draft exhibit; leftover figures are not decided numbers</t>
-        </is>
-      </c>
-      <c r="B1" s="62" t="n"/>
-      <c r="C1" s="62" t="n"/>
-      <c r="D1" s="62" t="n"/>
-      <c r="E1" s="62" t="n"/>
+          <t>ITEMS — Luke lock 3 Sep 2026. SET rows are closed. Yellow rows stay OPEN.</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Yellow commercial inputs on GC BID FORM and LANDIS FORM stay blank until these items are closed. Leftover figures below are from a prior template or an internal 8/21 note — they are not copied as bid values.</t>
+          <t>Closed by Luke on 3 Sep 2026: 21 weeks, $4,400/wk superintendent, 10% CM fee, 1.5% insurance, 1% pre-construction (first pay app / NTP). Leftover figures below are historical — SET rows use the locked number.</t>
         </is>
       </c>
     </row>
@@ -3234,102 +3323,102 @@
       </c>
     </row>
     <row r="4" ht="48" customHeight="1">
-      <c r="A4" s="65" t="n">
+      <c r="A4" s="116" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="66" t="inlineStr">
+      <c r="B4" s="117" t="inlineStr">
         <is>
           <t>Duration (weeks)</t>
         </is>
       </c>
-      <c r="C4" s="89" t="inlineStr">
-        <is>
-          <t>Leftover 13 weeks (prior Landis / super row) vs intake calendar 2027-04-02 to 2027-08-18 (~19.5 weeks). Mixed leftover payroll weeks on the old sheet were 24 / 7 / 13. None entered.</t>
-        </is>
-      </c>
-      <c r="D4" s="90" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E4" s="91" t="inlineStr">
-        <is>
-          <t>Luke / Landis</t>
+      <c r="C4" s="118" t="inlineStr">
+        <is>
+          <t>SET 21 weeks (Luke 3 Sep 2026). Intake calendar ~19.5 weeks (2027-04-02 to 2027-08-18). 20–23 week band reconciled at 21. Leftover 13 weeks not used.</t>
+        </is>
+      </c>
+      <c r="D4" s="119" t="inlineStr">
+        <is>
+          <t>SET</t>
+        </is>
+      </c>
+      <c r="E4" s="120" t="inlineStr">
+        <is>
+          <t>Luke</t>
         </is>
       </c>
     </row>
     <row r="5" ht="48" customHeight="1">
-      <c r="A5" s="65" t="n">
+      <c r="A5" s="116" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="66" t="inlineStr">
+      <c r="B5" s="117" t="inlineStr">
         <is>
           <t>Superintendent weekly rate</t>
         </is>
       </c>
-      <c r="C5" s="89" t="inlineStr">
-        <is>
-          <t>Leftover GC sheet $5,800/wk vs Shawn 8/21 $4,300/wk. Neither copied onto E49 or Landis E11.</t>
-        </is>
-      </c>
-      <c r="D5" s="90" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E5" s="91" t="inlineStr">
-        <is>
-          <t>Shawn</t>
+      <c r="C5" s="118" t="inlineStr">
+        <is>
+          <t>SET $4,400/wk (Luke 3 Sep 2026). Prior leftover $5,800 and Shawn 8/21 $4,300 superseded. On GC C-6.</t>
+        </is>
+      </c>
+      <c r="D5" s="119" t="inlineStr">
+        <is>
+          <t>SET</t>
+        </is>
+      </c>
+      <c r="E5" s="120" t="inlineStr">
+        <is>
+          <t>Luke</t>
         </is>
       </c>
     </row>
     <row r="6" ht="48" customHeight="1">
-      <c r="A6" s="65" t="n">
+      <c r="A6" s="116" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="66" t="inlineStr">
+      <c r="B6" s="117" t="inlineStr">
         <is>
           <t>CM fee / OH&amp;P %</t>
         </is>
       </c>
-      <c r="C6" s="89" t="inlineStr">
-        <is>
-          <t>Leftover 10% on prior GC A-1 vs Landis E12 blank. 10% not copied.</t>
-        </is>
-      </c>
-      <c r="D6" s="90" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E6" s="91" t="inlineStr">
+      <c r="C6" s="118" t="inlineStr">
+        <is>
+          <t>SET 10% (Luke 3 Sep 2026). Written to GC A-1 I33 and Landis E12.</t>
+        </is>
+      </c>
+      <c r="D6" s="119" t="inlineStr">
+        <is>
+          <t>SET</t>
+        </is>
+      </c>
+      <c r="E6" s="120" t="inlineStr">
         <is>
           <t>Luke</t>
         </is>
       </c>
     </row>
     <row r="7" ht="48" customHeight="1">
-      <c r="A7" s="65" t="n">
+      <c r="A7" s="116" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="66" t="inlineStr">
+      <c r="B7" s="117" t="inlineStr">
         <is>
           <t>Insurance %</t>
         </is>
       </c>
-      <c r="C7" s="89" t="inlineStr">
-        <is>
-          <t>Leftover 1.5% on prior GC B-3 vs Shawn 8/21 note 2%?. Neither copied onto I37 or Landis E13.</t>
-        </is>
-      </c>
-      <c r="D7" s="90" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E7" s="91" t="inlineStr">
-        <is>
-          <t>Shawn</t>
+      <c r="C7" s="118" t="inlineStr">
+        <is>
+          <t>SET 1.5% (Luke 3 Sep 2026; limits confirmed). Written to GC B-3 I37 and Landis E13. WC 1.2% stays on GC C-7 — not double-counted.</t>
+        </is>
+      </c>
+      <c r="D7" s="119" t="inlineStr">
+        <is>
+          <t>SET</t>
+        </is>
+      </c>
+      <c r="E7" s="120" t="inlineStr">
+        <is>
+          <t>Luke</t>
         </is>
       </c>
     </row>
@@ -3344,7 +3433,7 @@
       </c>
       <c r="C8" s="89" t="inlineStr">
         <is>
-          <t>Shawn 8/21: 4 trips × $1,500? (question mark). Prior sheet leftover $3,500/wk × 7 weeks. Weeks blank; trip price not entered as a decided number.</t>
+          <t>Still OPEN. Shawn 8/21: 4 trips × $1,500? Prior sheet leftover $3,500/wk × 7 weeks. Not invented. Job duration is 21 weeks; PM weeks/trips not filled.</t>
         </is>
       </c>
       <c r="D8" s="90" t="inlineStr">
@@ -3369,7 +3458,7 @@
       </c>
       <c r="C9" s="89" t="inlineStr">
         <is>
-          <t>Leftover 1% template on prior GC B-2. Not copied onto I36.</t>
+          <t>Template leftover 1% — not used. Not copied onto I36.</t>
         </is>
       </c>
       <c r="D9" s="90" t="inlineStr">
@@ -3387,6 +3476,163 @@
       <c r="A11" s="30" t="inlineStr">
         <is>
           <t>Color: yellow = OPEN. Owner is the person to close the item (Luke / Shawn / Landis). Calendar dates on COVER are intake facts, not a filled duration cell.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="121" t="n">
+        <v>7</v>
+      </c>
+      <c r="B12" s="121" t="inlineStr">
+        <is>
+          <t>Pre-construction fee</t>
+        </is>
+      </c>
+      <c r="C12" s="121" t="inlineStr">
+        <is>
+          <t>SET 1% of project total, payable with first pay application / NTP (not end of job). Dollar blank until trades are bid.</t>
+        </is>
+      </c>
+      <c r="D12" s="121" t="inlineStr">
+        <is>
+          <t>SET (rate) / OPEN (dollar)</t>
+        </is>
+      </c>
+      <c r="E12" s="121" t="inlineStr">
+        <is>
+          <t>Luke</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="122" t="n">
+        <v>8</v>
+      </c>
+      <c r="B13" s="122" t="inlineStr">
+        <is>
+          <t>CO markup %</t>
+        </is>
+      </c>
+      <c r="C13" s="122" t="inlineStr">
+        <is>
+          <t>Separate line. Not set. Do not assume equal to the 10% project CM fee. Landis E15 left blank.</t>
+        </is>
+      </c>
+      <c r="D13" s="122" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E13" s="122" t="inlineStr">
+        <is>
+          <t>Luke</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="122" t="n">
+        <v>9</v>
+      </c>
+      <c r="B14" s="122" t="inlineStr">
+        <is>
+          <t>Weekly GC lump</t>
+        </is>
+      </c>
+      <c r="C14" s="122" t="inlineStr">
+        <is>
+          <t>Still a weekly lump with breakouts. Super $4,400 SET. Do not invent a combined weekly GC dollar (PM still OPEN).</t>
+        </is>
+      </c>
+      <c r="D14" s="122" t="inlineStr">
+        <is>
+          <t>OPEN (lump)</t>
+        </is>
+      </c>
+      <c r="E14" s="122" t="inlineStr">
+        <is>
+          <t>Luke</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="122" t="n">
+        <v>10</v>
+      </c>
+      <c r="B15" s="122" t="inlineStr">
+        <is>
+          <t>Parking months / sprinkler shutdown count</t>
+        </is>
+      </c>
+      <c r="C15" s="122" t="inlineStr">
+        <is>
+          <t>Unit rates listed ($250/mo, $250 each). Counts not filled. Do not invent from 21 weeks.</t>
+        </is>
+      </c>
+      <c r="D15" s="122" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E15" s="122" t="inlineStr">
+        <is>
+          <t>Shawn / Landis</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="122" t="n">
+        <v>11</v>
+      </c>
+      <c r="B16" s="122" t="inlineStr">
+        <is>
+          <t>Grand total / trade packages</t>
+        </is>
+      </c>
+      <c r="C16" s="122" t="inlineStr">
+        <is>
+          <t>Packages 1–20 stay $0. Grand total depends on unbid trades. Not invented.</t>
+        </is>
+      </c>
+      <c r="D16" s="122" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E16" s="122" t="inlineStr">
+        <is>
+          <t>Bids</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="122" t="n">
+        <v>12</v>
+      </c>
+      <c r="B17" s="122" t="inlineStr">
+        <is>
+          <t>Net 90 vs net 45</t>
+        </is>
+      </c>
+      <c r="C17" s="122" t="inlineStr">
+        <is>
+          <t>Ralph Lauren payment policy is net 90. LBC standard is net 45. Gap still noted, not closed.</t>
+        </is>
+      </c>
+      <c r="D17" s="122" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E17" s="122" t="inlineStr">
+        <is>
+          <t>Luke / Charrette</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Blue-gray = SET (Luke 3 Sep 2026). Yellow = OPEN. Calendar dates on COVER are intake facts. Fee-form duration is 21 weeks.</t>
         </is>
       </c>
     </row>
@@ -3695,11 +3941,11 @@
           <t>Excluded / invoiced separately. Not extended on this sheet.</t>
         </is>
       </c>
-      <c r="D14" s="102" t="n"/>
-      <c r="E14" s="102" t="n"/>
-      <c r="F14" s="102" t="n"/>
-      <c r="G14" s="102" t="n"/>
-      <c r="H14" s="102" t="n"/>
+      <c r="D14" s="109" t="n"/>
+      <c r="E14" s="109" t="n"/>
+      <c r="F14" s="109" t="n"/>
+      <c r="G14" s="109" t="n"/>
+      <c r="H14" s="110" t="n"/>
     </row>
     <row r="15">
       <c r="B15" s="100" t="inlineStr">
@@ -3712,16 +3958,16 @@
           <t>Invoiced separately. Not extended on this sheet.</t>
         </is>
       </c>
-      <c r="D15" s="102" t="n"/>
-      <c r="E15" s="102" t="n"/>
-      <c r="F15" s="102" t="n"/>
-      <c r="G15" s="102" t="n"/>
-      <c r="H15" s="102" t="n"/>
+      <c r="D15" s="109" t="n"/>
+      <c r="E15" s="109" t="n"/>
+      <c r="F15" s="109" t="n"/>
+      <c r="G15" s="109" t="n"/>
+      <c r="H15" s="110" t="n"/>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="B17" s="103" t="inlineStr">
         <is>
-          <t>No job grand total is shown. Parking months and sprinkler-shutdown count stay OPEN. GC BID FORM D-22 (J76) remains $0 until mall fees are confirmed and entered. Green extensions are listed-rate × known qty only.</t>
+          <t>No job grand total is shown. Parking months and sprinkler-shutdown count stay OPEN (do not invent from 21 weeks). GC BID FORM D-22 (J76) remains $0 until mall fees are confirmed and entered. Green extensions are listed-rate × known qty only.</t>
         </is>
       </c>
     </row>
@@ -3820,7 +4066,7 @@
       </c>
       <c r="E5" s="105" t="inlineStr">
         <is>
-          <t>Not awarded.</t>
+          <t>Proposed, not awarded. Weekly rate set $4,400 (Luke 3 Sep 2026).</t>
         </is>
       </c>
     </row>

</xml_diff>